<commit_message>
Extend synthetic fixtures until every 02 rule and 04 quality path is exercised
New workbooks: SYN_D (alternate-only; text, dash, and negative prices; unpaired Unit Price column; stray row after a blank gap), SYN_E to SYN_H (persist into run 2 with one change each). Run 2 also replaces the award list and crosswalk. 04's Delta report now shows every status: NEW, REMOVED, CHANGED rows, CHANGED bidders, AWARDED, UNMAPPED, unchanged. A contractor row now carries price_suspicious_flag into the default mart.

Snapshots regenerated from the reference notebooks; refactored pipeline still matches them exactly (Gate 2a). tests/golden/test_path_coverage.py pins each path to snapshot evidence, since SQL and UDF paths are invisible to Python coverage. Coverage of src/bidtab_pipeline: line 92.9% -> 95.4%, branch 78.0% -> 82.7%. Backlog B-10: single-bidder workbooks are skipped. Adds pytest-cov to dev dependencies.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/config_synthetic/AwardedBidsSearchList.xlsx
+++ b/tests/fixtures/config_synthetic/AwardedBidsSearchList.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,6 +549,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2099-00007</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Synthetic G</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>India Co</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>700</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>